<commit_message>
feat(etf): update active ETF holdings for 20260921 and fix comparison sheet hyperlinks
- Fetch 31 active ETFs with 1,801 holdings for 20260921
- Update daily stock total sheet, top 10 addition/reduction charts, and dashboard_data.js
- Fix update_comparison_xlsx in collect_active_etf_holdings.py to preserve MoneyDJ hyperlinks and blue underline style
- Update handoff.md, docs/PROGRESS.md, and Obsidian daily note

handoff: updated 20260921 active ETF holdings, next: 20260922 daily update
</commit_message>
<xml_diff>
--- a/wiki/金融投資/台灣ETF比較清單.xlsx
+++ b/wiki/金融投資/台灣ETF比較清單.xlsx
@@ -2,8 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13140" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="主動型" sheetId="1" state="visible" r:id="rId1"/>
@@ -12,45 +13,24 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="槓桿反向" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="海外型" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'主動型'!$A$1:$H$33</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'市值型'!$A$1:$I$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'高股息'!$A$1:$I$22</definedName>
-  </definedNames>
-  <calcPr calcId="0" fullCalcOnLoad="1"/>
+  <definedNames/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="2">
     <font>
-      <name val="新細明體"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="新細明體"/>
-      <charset val="136"/>
-      <family val="3"/>
-      <sz val="9"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="新細明體"/>
-      <charset val="136"/>
-      <family val="1"/>
-      <color rgb="FF0563C1"/>
-      <sz val="11"/>
-      <u val="single"/>
-    </font>
-    <font>
-      <name val="新細明體"/>
       <color rgb="000563C1"/>
-      <sz val="11"/>
       <u val="single"/>
     </font>
   </fonts>
@@ -74,18 +54,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="1" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="一般" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -449,14 +423,16 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:H32"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15.75"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10.28515625" bestFit="1" customWidth="1" min="1" max="1"/>
-    <col width="22.28515625" bestFit="1" customWidth="1" min="2" max="2"/>
-    <col width="15.140625" bestFit="1" customWidth="1" min="3" max="4"/>
-    <col width="17.42578125" bestFit="1" customWidth="1" min="5" max="5"/>
-    <col width="15" bestFit="1" customWidth="1" min="6" max="7"/>
-    <col width="15.140625" bestFit="1" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -502,7 +478,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>00400A</t>
         </is>
@@ -544,7 +520,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" s="1" t="inlineStr">
         <is>
           <t>00401A</t>
         </is>
@@ -586,7 +562,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="1" t="inlineStr">
         <is>
           <t>00402A</t>
         </is>
@@ -628,7 +604,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="A5" s="1" t="inlineStr">
         <is>
           <t>00403A</t>
         </is>
@@ -670,7 +646,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="1" t="inlineStr">
         <is>
           <t>00404A</t>
         </is>
@@ -712,7 +688,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="A7" s="1" t="inlineStr">
         <is>
           <t>00405A</t>
         </is>
@@ -754,7 +730,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="A8" s="1" t="inlineStr">
         <is>
           <t>00406A</t>
         </is>
@@ -796,7 +772,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="A9" s="1" t="inlineStr">
         <is>
           <t>00407A</t>
         </is>
@@ -838,7 +814,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="inlineStr">
+      <c r="A10" s="1" t="inlineStr">
         <is>
           <t>00408A</t>
         </is>
@@ -880,7 +856,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+      <c r="A11" s="1" t="inlineStr">
         <is>
           <t>00980A</t>
         </is>
@@ -922,7 +898,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="inlineStr">
+      <c r="A12" s="1" t="inlineStr">
         <is>
           <t>00981A</t>
         </is>
@@ -964,7 +940,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr">
+      <c r="A13" s="1" t="inlineStr">
         <is>
           <t>00982A</t>
         </is>
@@ -1006,7 +982,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="inlineStr">
+      <c r="A14" s="1" t="inlineStr">
         <is>
           <t>00983A</t>
         </is>
@@ -1048,7 +1024,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="inlineStr">
+      <c r="A15" s="1" t="inlineStr">
         <is>
           <t>00984A</t>
         </is>
@@ -1090,7 +1066,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="inlineStr">
+      <c r="A16" s="1" t="inlineStr">
         <is>
           <t>00985A</t>
         </is>
@@ -1132,7 +1108,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="3" t="inlineStr">
+      <c r="A17" s="1" t="inlineStr">
         <is>
           <t>00986A</t>
         </is>
@@ -1174,7 +1150,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="inlineStr">
+      <c r="A18" s="1" t="inlineStr">
         <is>
           <t>00987A</t>
         </is>
@@ -1216,7 +1192,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="inlineStr">
+      <c r="A19" s="1" t="inlineStr">
         <is>
           <t>00988A</t>
         </is>
@@ -1258,7 +1234,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="3" t="inlineStr">
+      <c r="A20" s="1" t="inlineStr">
         <is>
           <t>00989A</t>
         </is>
@@ -1300,7 +1276,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="3" t="inlineStr">
+      <c r="A21" s="1" t="inlineStr">
         <is>
           <t>00990A</t>
         </is>
@@ -1342,7 +1318,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="3" t="inlineStr">
+      <c r="A22" s="1" t="inlineStr">
         <is>
           <t>00991A</t>
         </is>
@@ -1384,7 +1360,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="3" t="inlineStr">
+      <c r="A23" s="1" t="inlineStr">
         <is>
           <t>00992A</t>
         </is>
@@ -1426,7 +1402,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="3" t="inlineStr">
+      <c r="A24" s="1" t="inlineStr">
         <is>
           <t>00993A</t>
         </is>
@@ -1468,7 +1444,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="3" t="inlineStr">
+      <c r="A25" s="1" t="inlineStr">
         <is>
           <t>00994A</t>
         </is>
@@ -1510,7 +1486,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="3" t="inlineStr">
+      <c r="A26" s="1" t="inlineStr">
         <is>
           <t>00995A</t>
         </is>
@@ -1552,7 +1528,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="3" t="inlineStr">
+      <c r="A27" s="1" t="inlineStr">
         <is>
           <t>00996A</t>
         </is>
@@ -1594,7 +1570,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="3" t="inlineStr">
+      <c r="A28" s="1" t="inlineStr">
         <is>
           <t>00997A</t>
         </is>
@@ -1636,7 +1612,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="3" t="inlineStr">
+      <c r="A29" s="1" t="inlineStr">
         <is>
           <t>00998A</t>
         </is>
@@ -1678,7 +1654,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="3" t="inlineStr">
+      <c r="A30" s="1" t="inlineStr">
         <is>
           <t>00999A</t>
         </is>
@@ -1720,7 +1696,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="3" t="inlineStr">
+      <c r="A31" s="1" t="inlineStr">
         <is>
           <t>00980D</t>
         </is>
@@ -1762,7 +1738,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="3" t="inlineStr">
+      <c r="A32" s="1" t="inlineStr">
         <is>
           <t>00983D</t>
         </is>
@@ -1804,7 +1780,6 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H33"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A3" r:id="rId2"/>
@@ -1839,7 +1814,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A32" r:id="rId31"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="portrait" paperSize="9"/>
 </worksheet>
 </file>
 
@@ -1850,16 +1824,17 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I20"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15.75"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10.28515625" bestFit="1" customWidth="1" min="1" max="1"/>
-    <col width="20" bestFit="1" customWidth="1" min="2" max="2"/>
-    <col width="8.140625" bestFit="1" customWidth="1" min="3" max="3"/>
-    <col width="10.28515625" bestFit="1" customWidth="1" min="4" max="4"/>
-    <col width="29.42578125" bestFit="1" customWidth="1" min="5" max="5"/>
-    <col width="17.42578125" bestFit="1" customWidth="1" min="6" max="6"/>
-    <col width="15" bestFit="1" customWidth="1" min="7" max="8"/>
-    <col width="15.140625" bestFit="1" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="5" customWidth="1" min="3" max="3"/>
+    <col width="6" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1952,7 +1927,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026/07/21</t>
+          <t>2026/07/20</t>
         </is>
       </c>
     </row>
@@ -1999,7 +1974,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026/04/20</t>
+          <t>2026/04/17</t>
         </is>
       </c>
     </row>
@@ -2046,7 +2021,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026/10/22</t>
+          <t>2025/10/22</t>
         </is>
       </c>
     </row>
@@ -2093,7 +2068,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026/07/16</t>
+          <t>2026/07/15</t>
         </is>
       </c>
     </row>
@@ -2140,7 +2115,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026/07/16</t>
+          <t>2026/07/15</t>
         </is>
       </c>
     </row>
@@ -2187,7 +2162,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026/04/20</t>
+          <t>2026/04/17</t>
         </is>
       </c>
     </row>
@@ -2234,7 +2209,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026/08/21</t>
+          <t>2026/05/21</t>
         </is>
       </c>
     </row>
@@ -2281,7 +2256,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026/08/18</t>
+          <t>2026/01/19</t>
         </is>
       </c>
     </row>
@@ -2328,7 +2303,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026/07/27</t>
+          <t>2026/07/24</t>
         </is>
       </c>
     </row>
@@ -2375,7 +2350,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026/07/16</t>
+          <t>2026/07/15</t>
         </is>
       </c>
     </row>
@@ -2422,7 +2397,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2026/07/16</t>
+          <t>2026/07/15</t>
         </is>
       </c>
     </row>
@@ -2469,7 +2444,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2026/08/18</t>
+          <t>2026/02/26</t>
         </is>
       </c>
     </row>
@@ -2516,7 +2491,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>2026/06/16</t>
+          <t>2026/06/15</t>
         </is>
       </c>
     </row>
@@ -2563,7 +2538,7 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2026/03/17</t>
+          <t>2026/03/16</t>
         </is>
       </c>
     </row>
@@ -2610,7 +2585,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>2026/08/18</t>
+          <t>2026/02/25</t>
         </is>
       </c>
     </row>
@@ -2657,7 +2632,7 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>2026/03/17</t>
+          <t>2026/03/16</t>
         </is>
       </c>
     </row>
@@ -2704,7 +2679,7 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>2026/07/15</t>
+          <t>2026/07/14</t>
         </is>
       </c>
     </row>
@@ -2803,7 +2778,6 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I21"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A3" r:id="rId2"/>
@@ -2826,7 +2800,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A20" r:id="rId19"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="portrait" paperSize="9"/>
 </worksheet>
 </file>
 
@@ -2837,16 +2810,17 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I22"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15.75"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10.28515625" bestFit="1" customWidth="1" min="1" max="1"/>
-    <col width="24.7109375" bestFit="1" customWidth="1" min="2" max="2"/>
-    <col width="10.28515625" bestFit="1" customWidth="1" min="3" max="3"/>
-    <col width="15.140625" bestFit="1" customWidth="1" min="4" max="4"/>
-    <col width="31.85546875" bestFit="1" customWidth="1" min="5" max="5"/>
-    <col width="22.28515625" bestFit="1" customWidth="1" min="6" max="6"/>
-    <col width="15" bestFit="1" customWidth="1" min="7" max="8"/>
-    <col width="15.140625" bestFit="1" customWidth="1" min="9" max="9"/>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="6" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="21" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2939,7 +2913,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026/07/21</t>
+          <t>2026/07/20</t>
         </is>
       </c>
     </row>
@@ -2986,7 +2960,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026/08/18</t>
+          <t>2026/01/19</t>
         </is>
       </c>
     </row>
@@ -3033,7 +3007,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026/06/22</t>
+          <t>2026/06/18</t>
         </is>
       </c>
     </row>
@@ -3080,7 +3054,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026/08/18</t>
+          <t>2026/07/15</t>
         </is>
       </c>
     </row>
@@ -3127,7 +3101,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026/08/19</t>
+          <t>2026/05/19</t>
         </is>
       </c>
     </row>
@@ -3174,7 +3148,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026/08/18</t>
+          <t>2026/05/18</t>
         </is>
       </c>
     </row>
@@ -3221,7 +3195,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026/08/18</t>
+          <t>2026/07/15</t>
         </is>
       </c>
     </row>
@@ -3268,7 +3242,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026/08/25</t>
+          <t>2026/06/23</t>
         </is>
       </c>
     </row>
@@ -3315,7 +3289,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026/06/16</t>
+          <t>2026/06/15</t>
         </is>
       </c>
     </row>
@@ -3362,7 +3336,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026/06/18</t>
+          <t>2026/06/17</t>
         </is>
       </c>
     </row>
@@ -3409,7 +3383,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2026/06/16</t>
+          <t>2026/06/15</t>
         </is>
       </c>
     </row>
@@ -3456,7 +3430,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2026/08/19</t>
+          <t>2026/07/20</t>
         </is>
       </c>
     </row>
@@ -3503,7 +3477,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>2026/07/27</t>
+          <t>2026/07/24</t>
         </is>
       </c>
     </row>
@@ -3550,7 +3524,7 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2026/08/18</t>
+          <t>2026/07/15</t>
         </is>
       </c>
     </row>
@@ -3597,7 +3571,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>不配息</t>
+          <t>2026/07/14</t>
         </is>
       </c>
     </row>
@@ -3644,7 +3618,7 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>2026/07/02</t>
+          <t>2026/07/01</t>
         </is>
       </c>
     </row>
@@ -3691,7 +3665,7 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>2026/08/11</t>
+          <t>2026/07/08</t>
         </is>
       </c>
     </row>
@@ -3738,7 +3712,7 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>2026/08/18</t>
+          <t>2026/07/15</t>
         </is>
       </c>
     </row>
@@ -3785,7 +3759,7 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>2026/08/04</t>
+          <t>2026/07/03</t>
         </is>
       </c>
     </row>
@@ -3832,7 +3806,7 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>2026/08/18</t>
+          <t>2026/07/15</t>
         </is>
       </c>
     </row>
@@ -3879,12 +3853,11 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>2026/08/18</t>
+          <t>2026/07/15</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I22"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A3" r:id="rId2"/>
@@ -3919,14 +3892,15 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G12"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15.75"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10.28515625" bestFit="1" customWidth="1" min="1" max="1"/>
-    <col width="18.7109375" bestFit="1" customWidth="1" min="2" max="2"/>
-    <col width="30.42578125" bestFit="1" customWidth="1" min="3" max="3"/>
-    <col width="8.140625" bestFit="1" customWidth="1" min="4" max="4"/>
-    <col width="10.28515625" bestFit="1" customWidth="1" min="5" max="5"/>
-    <col width="15" bestFit="1" customWidth="1" min="6" max="7"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="5" customWidth="1" min="4" max="4"/>
+    <col width="6" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4397,18 +4371,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.5703125" defaultRowHeight="15.75"/>
+  <dimension ref="A1:H13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10.28515625" bestFit="1" customWidth="1" min="1" max="1"/>
-    <col width="29" bestFit="1" customWidth="1" min="2" max="2"/>
-    <col width="33.85546875" bestFit="1" customWidth="1" min="3" max="3"/>
-    <col width="8.140625" bestFit="1" customWidth="1" min="4" max="4"/>
-    <col width="20" bestFit="1" customWidth="1" min="5" max="5"/>
-    <col width="15.28515625" bestFit="1" customWidth="1" min="6" max="6"/>
-    <col width="15" bestFit="1" customWidth="1" min="7" max="7"/>
-    <col width="20.85546875" bestFit="1" customWidth="1" min="8" max="8"/>
-    <col width="15.140625" bestFit="1" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="5" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4452,11 +4425,6 @@
           <t>保管費 (年率)</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>最近除息日期</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
@@ -4499,11 +4467,6 @@
           <t>0.06% (級距)</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>不配息</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
@@ -4546,11 +4509,6 @@
           <t>0.16%~0.21%</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>不配息</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
@@ -4593,11 +4551,6 @@
           <t>0.08%~0.16%</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>2026/06/17</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
@@ -4640,11 +4593,6 @@
           <t>0.18%</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>不配息</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
@@ -4687,11 +4635,6 @@
           <t>0.10%~0.15%</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>2026/01/20</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
@@ -4734,11 +4677,6 @@
           <t>0.06%~0.11%</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>2026/01/20</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
@@ -4781,11 +4719,6 @@
           <t>0.08%~0.15%</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>不配息</t>
-        </is>
-      </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
@@ -4828,162 +4761,142 @@
           <t>0.20%</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>不配息</t>
-        </is>
-      </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>009821</t>
+          <t>009823</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>野村全球稀土與關鍵資源</t>
+          <t>群益標普500 ETF</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>張怡琳</t>
+          <t>標普 500 指數（S&amp;P 500 Index）</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>永豐商業銀行</t>
+          <t>謝明志</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>NYSE TIP全球稀土與關鍵資源指數</t>
+          <t>華南銀行</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>不配息</t>
+          <t>季配 (2,5,8,11)</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>0.90%</t>
+          <t>0.20% (級距)</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>0.20%</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>不配息</t>
+          <t>0.06%~0.10% (級距)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>009823</t>
+          <t>009824</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>群益標普500 ETF</t>
+          <t>群益美國科技巨頭ETF基金</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>標普 500 指數（S&amp;P 500 Index）</t>
+          <t>Solactive美國科技巨頭指數</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>謝明志</t>
+          <t>李晉含</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>華南銀行</t>
+          <t>中國信託商業銀行</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>季配 (2,5,8,11)</t>
+          <t>季配 (3,6,9,12)</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>0.20% (級距)</t>
+          <t>0.80%</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>0.06%~0.10% (級距)</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>尚未除息</t>
+          <t>0.06%~0.12% (級距)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>009824</t>
+          <t>009821</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>群益美國科技巨頭ETF基金</t>
+          <t>野村全球稀土與關鍵資源</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Solactive美國科技巨頭指數</t>
+          <t>NYSE TIP全球稀土與關鍵資源指數</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>李晉含</t>
+          <t>張怡琳</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>中國信託商業銀行</t>
+          <t>永豐商業銀行</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>季配 (3,6,9,12)</t>
+          <t>不配息</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>0.80%</t>
+          <t>0.90%</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>0.06%~0.12% (級距)</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>尚未除息</t>
+          <t>0.20%</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+      <c r="A13" s="1" t="inlineStr">
         <is>
           <t>009826</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>貝萊德iShares安碩世界股票</t>
+          <t>貝萊德iShares未來世界股票</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -4998,7 +4911,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>渣打銀行</t>
+          <t>華南商業銀行</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -5008,17 +4921,12 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>0.40%~0.45%</t>
+          <t>0.75%</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>0.10%~0.15%</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>不配息</t>
+          <t>0.15%</t>
         </is>
       </c>
     </row>

</xml_diff>